<commit_message>
User story backlog: acceptance criteria of a merged story carry their FR with the AC number; epic FR lists without repeats
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Backlog/BIBS_Backlog_BRD-00_User_Story_Backlog_Drop-0_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Backlog/BIBS_Backlog_BRD-00_User_Story_Backlog_Drop-0_v1.0.xlsx
@@ -43861,8 +43861,8 @@
       </c>
       <c r="P45" s="12" t="inlineStr">
         <is>
-          <t>(AC1) Given the user has UAM_REPORT_VIEW and the Marketing Account Officer profile, when the user selects the report, the profile(s), area and active flag, then the report lists Client Management tasks with "With Access" or "No Access".
-(AC1) Given the user has UAM_REPORT_VIEW, when the user selects the report, the profile(s) and the as-of date, then the list shows every member of Marketing Team Lead with the user who added each member and the date.</t>
+          <t>(FR-UA-061 AC1) Given the user has UAM_REPORT_VIEW and the Marketing Account Officer profile, when the user selects the report, the profile(s), area and active flag, then the report lists Client Management tasks with "With Access" or "No Access".
+(FR-UA-062 AC1) Given the user has UAM_REPORT_VIEW, when the user selects the report, the profile(s) and the as-of date, then the list shows every member of Marketing Team Lead with the user who added each member and the date.</t>
         </is>
       </c>
       <c r="Q45" s="12" t="inlineStr">
@@ -43898,8 +43898,8 @@
 *Business rules*
 * (R1) Module and task come from the permission areas and action classes; the BRD sample's QPS task names are UQ11. (Fixed)
 *Acceptance criteria*
-* (AC1) Given the user has UAM_REPORT_VIEW and the Marketing Account Officer profile, when the user selects the report, the profile(s), area and active flag, then the report lists Client Management tasks with "With Access" or "No Access".
-* (AC1) Given the user has UAM_REPORT_VIEW, when the user selects the report, the profile(s) and the as-of date, then the list shows every member of Marketing Team Lead with the user who added each member and the date.
+* (FR-UA-061 AC1) Given the user has UAM_REPORT_VIEW and the Marketing Account Officer profile, when the user selects the report, the profile(s), area and active flag, then the report lists Client Management tasks with "With Access" or "No Access".
+* (FR-UA-062 AC1) Given the user has UAM_REPORT_VIEW, when the user selects the report, the profile(s) and the as-of date, then the list shows every member of Marketing Team Lead with the user who added each member and the date.
 *Out of scope / notes*
 * CLR-UA-10 - open, for BDOI confirmation: Module and task names in the reports (3.003; FR-UA-060, 061). Proposed: The User Group Profile Report shows the module as the permission area and the task as the permission name. The report parameters Group Profile and Module are offered as lists. Decision requested: Confirm the module and task names (UQ11, UA-Q50).
 * FR-UA-061 and FR-UA-062 are one story: each has one acceptance criterion on the same screen.
@@ -46819,7 +46819,7 @@
       </c>
       <c r="M22" s="12" t="inlineStr">
         <is>
-          <t>FR-DM-030, FR-DM-031, FR-DM-032, FR-DM-033, FR-DM-034, FR-DM-034</t>
+          <t>FR-DM-030, FR-DM-031, FR-DM-032, FR-DM-033, FR-DM-034</t>
         </is>
       </c>
       <c r="N22" s="12" t="inlineStr"/>
@@ -46835,7 +46835,7 @@
       <c r="T22" s="12" t="inlineStr">
         <is>
           <t>Capability Client master and reference data of Data Migration (BRD-13): section 20.4 of the Data Migration Handbook BRD-13 Data Migration v2.1 (02_BIBS_Handbook_BRD-13_Data_Migration_v2.1.docx).
-Stories: 6, story points (first estimate): 20. FRs: FR-DM-030, FR-DM-031, FR-DM-032, FR-DM-033, FR-DM-034, FR-DM-034.
+Stories: 6, story points (first estimate): 20. FRs: FR-DM-030, FR-DM-031, FR-DM-032, FR-DM-033, FR-DM-034.
 Fix version: Drop 0.</t>
         </is>
       </c>

</xml_diff>